<commit_message>
Fix Geelong rating flip, add CSAT chart, rename analysis doc
- clean.py: invert Geelong ratings on the 2025 sheet only (2026 uses 5 = best); rerun cleaning and update ratings in AI outputs
- Add CSAT by dealership chart (00) and stats; overall customer satisfaction section in business answers
- Rename business answers to Dealer Customer Satisfaction Performance Analysis; remove department chart (08)
- Add root-cause, initial observations, AI model/API rationale and reflection notes to the reports
</commit_message>
<xml_diff>
--- a/code_and_data/ai_output/management_summary.xlsx
+++ b/code_and_data/ai_output/management_summary.xlsx
@@ -16003,7 +16003,6 @@
           <t>Service</t>
         </is>
       </c>
-      <c r="G189" t="inlineStr"/>
       <c r="H189" t="inlineStr">
         <is>
           <t>Repair &amp; Service Quality</t>
@@ -16374,7 +16373,6 @@
           <t>Service</t>
         </is>
       </c>
-      <c r="G194" t="inlineStr"/>
       <c r="H194" t="inlineStr">
         <is>
           <t>Parts Availability &amp; Delays</t>
@@ -32742,7 +32740,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>319</v>
+        <v>311</v>
       </c>
     </row>
     <row r="4">
@@ -32762,7 +32760,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>227</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6">
@@ -32772,7 +32770,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>222</v>
+        <v>196</v>
       </c>
     </row>
     <row r="7">
@@ -32782,7 +32780,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>185</v>
+        <v>193</v>
       </c>
     </row>
     <row r="8">
@@ -32792,27 +32790,27 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Vehicle Knowledge &amp; Explanation</t>
+          <t>Safety Concern</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Safety Concern</t>
+          <t>Vehicle Knowledge &amp; Explanation</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>104</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11">
@@ -32822,7 +32820,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>79</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12">
@@ -32832,7 +32830,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13">
@@ -32842,7 +32840,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14">

</xml_diff>